<commit_message>
Add data for historical-policy-parameters branch
</commit_message>
<xml_diff>
--- a/captax/data/outputs/Current-Law/comprehensive/supplemental_table_EMTRs_Current-Law_comprehensive.xlsx
+++ b/captax/data/outputs/Current-Law/comprehensive/supplemental_table_EMTRs_Current-Law_comprehensive.xlsx
@@ -474,24 +474,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A5:M45"/>
+  <dimension ref="A5:V45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="65.7109375" customWidth="1"/>
-    <col min="2" max="13" width="9.7109375" style="1" customWidth="1"/>
+    <col min="2" max="22" width="9.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:21">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:21">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:21">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -504,43 +504,79 @@
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
-    </row>
-    <row r="9" spans="1:12">
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+    </row>
+    <row r="9" spans="1:21">
       <c r="B9" s="5">
+        <v>2016</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2017</v>
+      </c>
+      <c r="D9" s="5">
+        <v>2018</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2019</v>
+      </c>
+      <c r="F9" s="5">
+        <v>2020</v>
+      </c>
+      <c r="G9" s="5">
+        <v>2021</v>
+      </c>
+      <c r="H9" s="5">
+        <v>2022</v>
+      </c>
+      <c r="I9" s="5">
+        <v>2023</v>
+      </c>
+      <c r="J9" s="5">
+        <v>2024</v>
+      </c>
+      <c r="K9" s="5">
         <v>2025</v>
       </c>
-      <c r="C9" s="5">
+      <c r="L9" s="5">
         <v>2026</v>
       </c>
-      <c r="D9" s="5">
+      <c r="M9" s="5">
         <v>2027</v>
       </c>
-      <c r="E9" s="5">
+      <c r="N9" s="5">
         <v>2028</v>
       </c>
-      <c r="F9" s="5">
+      <c r="O9" s="5">
         <v>2029</v>
       </c>
-      <c r="G9" s="5">
+      <c r="P9" s="5">
         <v>2030</v>
       </c>
-      <c r="H9" s="5">
+      <c r="Q9" s="5">
         <v>2031</v>
       </c>
-      <c r="I9" s="5">
+      <c r="R9" s="5">
         <v>2032</v>
       </c>
-      <c r="J9" s="5">
+      <c r="S9" s="5">
         <v>2033</v>
       </c>
-      <c r="K9" s="5">
+      <c r="T9" s="5">
         <v>2034</v>
       </c>
-      <c r="L9" s="5">
+      <c r="U9" s="5">
         <v>2035</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:21">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -553,760 +589,1282 @@
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
-    </row>
-    <row r="11" spans="1:12">
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+    </row>
+    <row r="11" spans="1:21">
       <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:21">
       <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="1">
+        <v>14.67</v>
+      </c>
+      <c r="C12" s="1">
+        <v>14.88</v>
+      </c>
+      <c r="D12" s="1">
+        <v>12.83</v>
+      </c>
+      <c r="E12" s="1">
+        <v>12.38</v>
+      </c>
+      <c r="F12" s="1">
+        <v>12.55</v>
+      </c>
+      <c r="G12" s="1">
+        <v>13.66</v>
+      </c>
+      <c r="H12" s="1">
+        <v>13.67</v>
+      </c>
+      <c r="I12" s="1">
+        <v>13.61</v>
+      </c>
+      <c r="J12" s="1">
+        <v>14.29</v>
+      </c>
+      <c r="K12" s="1">
         <v>14.74</v>
       </c>
-      <c r="C12" s="1">
+      <c r="L12" s="1">
         <v>14.43</v>
       </c>
-      <c r="D12" s="1">
+      <c r="M12" s="1">
         <v>15.06</v>
       </c>
-      <c r="E12" s="1">
+      <c r="N12" s="1">
         <v>15.09</v>
       </c>
-      <c r="F12" s="1">
+      <c r="O12" s="1">
         <v>15.04</v>
       </c>
-      <c r="G12" s="1">
+      <c r="P12" s="1">
         <v>15.18</v>
       </c>
-      <c r="H12" s="1">
+      <c r="Q12" s="1">
         <v>15.3</v>
       </c>
-      <c r="I12" s="1">
+      <c r="R12" s="1">
         <v>15.19</v>
       </c>
-      <c r="J12" s="1">
+      <c r="S12" s="1">
         <v>15.31</v>
       </c>
-      <c r="K12" s="1">
+      <c r="T12" s="1">
         <v>15.22</v>
       </c>
-      <c r="L12" s="1">
+      <c r="U12" s="1">
         <v>15.28</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:21">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="1">
+        <v>22.25</v>
+      </c>
+      <c r="C14" s="1">
+        <v>22.51</v>
+      </c>
+      <c r="D14" s="1">
+        <v>15.92</v>
+      </c>
+      <c r="E14" s="1">
+        <v>15.66</v>
+      </c>
+      <c r="F14" s="1">
+        <v>15.81</v>
+      </c>
+      <c r="G14" s="1">
+        <v>16.73</v>
+      </c>
+      <c r="H14" s="1">
+        <v>16.78</v>
+      </c>
+      <c r="I14" s="1">
+        <v>16.63</v>
+      </c>
+      <c r="J14" s="1">
+        <v>17.64</v>
+      </c>
+      <c r="K14" s="1">
         <v>18.5</v>
       </c>
-      <c r="C14" s="1">
+      <c r="L14" s="1">
         <v>21.28</v>
       </c>
-      <c r="D14" s="1">
+      <c r="M14" s="1">
         <v>22.28</v>
       </c>
-      <c r="E14" s="1">
+      <c r="N14" s="1">
         <v>22.36</v>
       </c>
-      <c r="F14" s="1">
+      <c r="O14" s="1">
         <v>22.38</v>
       </c>
-      <c r="G14" s="1">
+      <c r="P14" s="1">
         <v>22.57</v>
       </c>
-      <c r="H14" s="1">
+      <c r="Q14" s="1">
         <v>22.71</v>
       </c>
-      <c r="I14" s="1">
+      <c r="R14" s="1">
         <v>22.64</v>
       </c>
-      <c r="J14" s="1">
+      <c r="S14" s="1">
         <v>22.76</v>
       </c>
-      <c r="K14" s="1">
+      <c r="T14" s="1">
         <v>22.73</v>
       </c>
-      <c r="L14" s="1">
+      <c r="U14" s="1">
         <v>22.81</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:21">
       <c r="A15" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:21">
       <c r="A16" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B16" s="1">
+        <v>12.44</v>
+      </c>
+      <c r="C16" s="1">
+        <v>12.66</v>
+      </c>
+      <c r="D16" s="1">
+        <v>5.04</v>
+      </c>
+      <c r="E16" s="1">
+        <v>4.68</v>
+      </c>
+      <c r="F16" s="1">
+        <v>4.76</v>
+      </c>
+      <c r="G16" s="1">
+        <v>5.82</v>
+      </c>
+      <c r="H16" s="1">
+        <v>5.46</v>
+      </c>
+      <c r="I16" s="1">
+        <v>6.28</v>
+      </c>
+      <c r="J16" s="1">
+        <v>9.390000000000001</v>
+      </c>
+      <c r="K16" s="1">
         <v>12.12</v>
       </c>
-      <c r="C16" s="1">
+      <c r="L16" s="1">
         <v>15.49</v>
       </c>
-      <c r="D16" s="1">
+      <c r="M16" s="1">
         <v>18.65</v>
       </c>
-      <c r="E16" s="1">
+      <c r="N16" s="1">
         <v>18.8</v>
       </c>
-      <c r="F16" s="1">
+      <c r="O16" s="1">
         <v>18.97</v>
       </c>
-      <c r="G16" s="1">
+      <c r="P16" s="1">
         <v>19.32</v>
       </c>
-      <c r="H16" s="1">
+      <c r="Q16" s="1">
         <v>19.47</v>
       </c>
-      <c r="I16" s="1">
+      <c r="R16" s="1">
         <v>19.44</v>
       </c>
-      <c r="J16" s="1">
+      <c r="S16" s="1">
         <v>19.54</v>
       </c>
-      <c r="K16" s="1">
+      <c r="T16" s="1">
         <v>19.51</v>
       </c>
-      <c r="L16" s="1">
+      <c r="U16" s="1">
         <v>19.58</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:21">
       <c r="A17" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="1">
+        <v>25.98</v>
+      </c>
+      <c r="C17" s="1">
+        <v>26.25</v>
+      </c>
+      <c r="D17" s="1">
+        <v>19.72</v>
+      </c>
+      <c r="E17" s="1">
+        <v>19.52</v>
+      </c>
+      <c r="F17" s="1">
+        <v>19.65</v>
+      </c>
+      <c r="G17" s="1">
+        <v>20.55</v>
+      </c>
+      <c r="H17" s="1">
+        <v>19.93</v>
+      </c>
+      <c r="I17" s="1">
+        <v>19.68</v>
+      </c>
+      <c r="J17" s="1">
+        <v>20.31</v>
+      </c>
+      <c r="K17" s="1">
         <v>20.79</v>
       </c>
-      <c r="C17" s="1">
+      <c r="L17" s="1">
         <v>23.02</v>
       </c>
-      <c r="D17" s="1">
+      <c r="M17" s="1">
         <v>23.69</v>
       </c>
-      <c r="E17" s="1">
+      <c r="N17" s="1">
         <v>23.71</v>
       </c>
-      <c r="F17" s="1">
+      <c r="O17" s="1">
         <v>23.67</v>
       </c>
-      <c r="G17" s="1">
+      <c r="P17" s="1">
         <v>23.78</v>
       </c>
-      <c r="H17" s="1">
+      <c r="Q17" s="1">
         <v>23.9</v>
       </c>
-      <c r="I17" s="1">
+      <c r="R17" s="1">
         <v>23.8</v>
       </c>
-      <c r="J17" s="1">
+      <c r="S17" s="1">
         <v>23.95</v>
       </c>
-      <c r="K17" s="1">
+      <c r="T17" s="1">
         <v>23.89</v>
       </c>
-      <c r="L17" s="1">
+      <c r="U17" s="1">
         <v>23.98</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:21">
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B18" s="1">
+        <v>27.24</v>
+      </c>
+      <c r="C18" s="1">
+        <v>27.52</v>
+      </c>
+      <c r="D18" s="1">
+        <v>22.64</v>
+      </c>
+      <c r="E18" s="1">
+        <v>22.36</v>
+      </c>
+      <c r="F18" s="1">
+        <v>22.5</v>
+      </c>
+      <c r="G18" s="1">
+        <v>23.36</v>
+      </c>
+      <c r="H18" s="1">
+        <v>23.09</v>
+      </c>
+      <c r="I18" s="1">
+        <v>23.02</v>
+      </c>
+      <c r="J18" s="1">
+        <v>23.26</v>
+      </c>
+      <c r="K18" s="1">
         <v>23.47</v>
       </c>
-      <c r="C18" s="1">
+      <c r="L18" s="1">
         <v>27.26</v>
       </c>
-      <c r="D18" s="1">
+      <c r="M18" s="1">
         <v>27.38</v>
       </c>
-      <c r="E18" s="1">
+      <c r="N18" s="1">
         <v>27.43</v>
       </c>
-      <c r="F18" s="1">
+      <c r="O18" s="1">
         <v>27.26</v>
       </c>
-      <c r="G18" s="1">
+      <c r="P18" s="1">
         <v>27.23</v>
       </c>
-      <c r="H18" s="1">
+      <c r="Q18" s="1">
         <v>27.38</v>
       </c>
-      <c r="I18" s="1">
+      <c r="R18" s="1">
         <v>27.29</v>
       </c>
-      <c r="J18" s="1">
+      <c r="S18" s="1">
         <v>27.42</v>
       </c>
-      <c r="K18" s="1">
+      <c r="T18" s="1">
         <v>27.41</v>
       </c>
-      <c r="L18" s="1">
+      <c r="U18" s="1">
         <v>27.5</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:21">
       <c r="A19" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="1">
+        <v>-38.43</v>
+      </c>
+      <c r="C19" s="1">
+        <v>-38.15</v>
+      </c>
+      <c r="D19" s="1">
+        <v>-27.26</v>
+      </c>
+      <c r="E19" s="1">
+        <v>-27.77</v>
+      </c>
+      <c r="F19" s="1">
+        <v>-27.49</v>
+      </c>
+      <c r="G19" s="1">
+        <v>-26.09</v>
+      </c>
+      <c r="H19" s="1">
+        <v>-13.6</v>
+      </c>
+      <c r="I19" s="1">
+        <v>-18.28</v>
+      </c>
+      <c r="J19" s="1">
+        <v>-17.4</v>
+      </c>
+      <c r="K19" s="1">
         <v>-16.89</v>
       </c>
-      <c r="C19" s="1">
+      <c r="L19" s="1">
         <v>-15.38</v>
       </c>
-      <c r="D19" s="1">
+      <c r="M19" s="1">
         <v>-14.92</v>
       </c>
-      <c r="E19" s="1">
+      <c r="N19" s="1">
         <v>-14.29</v>
       </c>
-      <c r="F19" s="1">
+      <c r="O19" s="1">
         <v>-12.96</v>
       </c>
-      <c r="G19" s="1">
+      <c r="P19" s="1">
         <v>-11.22</v>
       </c>
-      <c r="H19" s="1">
+      <c r="Q19" s="1">
         <v>-10.93</v>
       </c>
-      <c r="I19" s="1">
+      <c r="R19" s="1">
         <v>-10.91</v>
       </c>
-      <c r="J19" s="1">
+      <c r="S19" s="1">
         <v>-10.8</v>
       </c>
-      <c r="K19" s="1">
+      <c r="T19" s="1">
         <v>-10.83</v>
       </c>
-      <c r="L19" s="1">
+      <c r="U19" s="1">
         <v>-10.75</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:21">
       <c r="A20" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="1">
+        <v>26.32</v>
+      </c>
+      <c r="C20" s="1">
+        <v>26.49</v>
+      </c>
+      <c r="D20" s="1">
+        <v>14.49</v>
+      </c>
+      <c r="E20" s="1">
+        <v>14.16</v>
+      </c>
+      <c r="F20" s="1">
+        <v>14.32</v>
+      </c>
+      <c r="G20" s="1">
+        <v>15.26</v>
+      </c>
+      <c r="H20" s="1">
+        <v>14.88</v>
+      </c>
+      <c r="I20" s="1">
+        <v>17.46</v>
+      </c>
+      <c r="J20" s="1">
+        <v>20.13</v>
+      </c>
+      <c r="K20" s="1">
         <v>22.46</v>
       </c>
-      <c r="C20" s="1">
+      <c r="L20" s="1">
         <v>25.33</v>
       </c>
-      <c r="D20" s="1">
+      <c r="M20" s="1">
         <v>27.35</v>
       </c>
-      <c r="E20" s="1">
+      <c r="N20" s="1">
         <v>27.44</v>
       </c>
-      <c r="F20" s="1">
+      <c r="O20" s="1">
         <v>27.5</v>
       </c>
-      <c r="G20" s="1">
+      <c r="P20" s="1">
         <v>27.7</v>
       </c>
-      <c r="H20" s="1">
+      <c r="Q20" s="1">
         <v>27.83</v>
       </c>
-      <c r="I20" s="1">
+      <c r="R20" s="1">
         <v>27.81</v>
       </c>
-      <c r="J20" s="1">
+      <c r="S20" s="1">
         <v>27.9</v>
       </c>
-      <c r="K20" s="1">
+      <c r="T20" s="1">
         <v>27.87</v>
       </c>
-      <c r="L20" s="1">
+      <c r="U20" s="1">
         <v>27.93</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:21">
       <c r="A21" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B21" s="1">
+        <v>37.61</v>
+      </c>
+      <c r="C21" s="1">
+        <v>37.77</v>
+      </c>
+      <c r="D21" s="1">
+        <v>29.02</v>
+      </c>
+      <c r="E21" s="1">
+        <v>28.76</v>
+      </c>
+      <c r="F21" s="1">
+        <v>29.02</v>
+      </c>
+      <c r="G21" s="1">
+        <v>29.74</v>
+      </c>
+      <c r="H21" s="1">
+        <v>29.42</v>
+      </c>
+      <c r="I21" s="1">
+        <v>29.09</v>
+      </c>
+      <c r="J21" s="1">
+        <v>29.32</v>
+      </c>
+      <c r="K21" s="1">
         <v>29.44</v>
       </c>
-      <c r="C21" s="1">
+      <c r="L21" s="1">
         <v>32.13</v>
       </c>
-      <c r="D21" s="1">
+      <c r="M21" s="1">
         <v>32.19</v>
       </c>
-      <c r="E21" s="1">
+      <c r="N21" s="1">
         <v>32.23</v>
       </c>
-      <c r="F21" s="1">
+      <c r="O21" s="1">
         <v>32.1</v>
       </c>
-      <c r="G21" s="1">
+      <c r="P21" s="1">
         <v>32.09</v>
       </c>
-      <c r="H21" s="1">
+      <c r="Q21" s="1">
         <v>32.23</v>
       </c>
-      <c r="I21" s="1">
+      <c r="R21" s="1">
         <v>32.19</v>
       </c>
-      <c r="J21" s="1">
+      <c r="S21" s="1">
         <v>32.28</v>
       </c>
-      <c r="K21" s="1">
+      <c r="T21" s="1">
         <v>32.28</v>
       </c>
-      <c r="L21" s="1">
+      <c r="U21" s="1">
         <v>32.36</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:21">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:21">
       <c r="A23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="1">
+        <v>28.71</v>
+      </c>
+      <c r="C23" s="1">
+        <v>28.84</v>
+      </c>
+      <c r="D23" s="1">
+        <v>19.25</v>
+      </c>
+      <c r="E23" s="1">
+        <v>19.17</v>
+      </c>
+      <c r="F23" s="1">
+        <v>19.43</v>
+      </c>
+      <c r="G23" s="1">
+        <v>19.75</v>
+      </c>
+      <c r="H23" s="1">
+        <v>19.87</v>
+      </c>
+      <c r="I23" s="1">
+        <v>19.99</v>
+      </c>
+      <c r="J23" s="1">
+        <v>20.87</v>
+      </c>
+      <c r="K23" s="1">
         <v>21.6</v>
       </c>
-      <c r="C23" s="1">
+      <c r="L23" s="1">
         <v>24.64</v>
       </c>
-      <c r="D23" s="1">
+      <c r="M23" s="1">
         <v>25.55</v>
       </c>
-      <c r="E23" s="1">
+      <c r="N23" s="1">
         <v>25.57</v>
       </c>
-      <c r="F23" s="1">
+      <c r="O23" s="1">
         <v>25.55</v>
       </c>
-      <c r="G23" s="1">
+      <c r="P23" s="1">
         <v>25.66</v>
       </c>
-      <c r="H23" s="1">
+      <c r="Q23" s="1">
         <v>25.78</v>
       </c>
-      <c r="I23" s="1">
+      <c r="R23" s="1">
         <v>25.75</v>
       </c>
-      <c r="J23" s="1">
+      <c r="S23" s="1">
         <v>25.84</v>
       </c>
-      <c r="K23" s="1">
+      <c r="T23" s="1">
         <v>25.86</v>
       </c>
-      <c r="L23" s="1">
+      <c r="U23" s="1">
         <v>25.92</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:21">
       <c r="A24" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B24" s="1">
+        <v>-17.81</v>
+      </c>
+      <c r="C24" s="1">
+        <v>-16.87</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.49</v>
+      </c>
+      <c r="E24" s="1">
+        <v>-0.75</v>
+      </c>
+      <c r="F24" s="1">
+        <v>-1.01</v>
+      </c>
+      <c r="G24" s="1">
+        <v>2.93</v>
+      </c>
+      <c r="H24" s="1">
+        <v>2.49</v>
+      </c>
+      <c r="I24" s="1">
+        <v>0.76</v>
+      </c>
+      <c r="J24" s="1">
+        <v>2.49</v>
+      </c>
+      <c r="K24" s="1">
         <v>3.96</v>
       </c>
-      <c r="C24" s="1">
+      <c r="L24" s="1">
         <v>4.68</v>
       </c>
-      <c r="D24" s="1">
+      <c r="M24" s="1">
         <v>6.24</v>
       </c>
-      <c r="E24" s="1">
+      <c r="N24" s="1">
         <v>6.62</v>
       </c>
-      <c r="F24" s="1">
+      <c r="O24" s="1">
         <v>6.94</v>
       </c>
-      <c r="G24" s="1">
+      <c r="P24" s="1">
         <v>7.55</v>
       </c>
-      <c r="H24" s="1">
+      <c r="Q24" s="1">
         <v>7.8</v>
       </c>
-      <c r="I24" s="1">
+      <c r="R24" s="1">
         <v>7.5</v>
       </c>
-      <c r="J24" s="1">
+      <c r="S24" s="1">
         <v>7.82</v>
       </c>
-      <c r="K24" s="1">
+      <c r="T24" s="1">
         <v>7.48</v>
       </c>
-      <c r="L24" s="1">
+      <c r="U24" s="1">
         <v>7.63</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:21">
       <c r="A25" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:21">
       <c r="A26" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B26" s="1">
+        <v>21.67</v>
+      </c>
+      <c r="C26" s="1">
+        <v>21.9</v>
+      </c>
+      <c r="D26" s="1">
+        <v>14.45</v>
+      </c>
+      <c r="E26" s="1">
+        <v>14.18</v>
+      </c>
+      <c r="F26" s="1">
+        <v>14.32</v>
+      </c>
+      <c r="G26" s="1">
+        <v>15.31</v>
+      </c>
+      <c r="H26" s="1">
+        <v>15.42</v>
+      </c>
+      <c r="I26" s="1">
+        <v>15.06</v>
+      </c>
+      <c r="J26" s="1">
+        <v>16.24</v>
+      </c>
+      <c r="K26" s="1">
         <v>17.17</v>
       </c>
-      <c r="C26" s="1">
+      <c r="L26" s="1">
         <v>18.55</v>
       </c>
-      <c r="D26" s="1">
+      <c r="M26" s="1">
         <v>19.69</v>
       </c>
-      <c r="E26" s="1">
+      <c r="N26" s="1">
         <v>19.79</v>
       </c>
-      <c r="F26" s="1">
+      <c r="O26" s="1">
         <v>19.92</v>
       </c>
-      <c r="G26" s="1">
+      <c r="P26" s="1">
         <v>20.22</v>
       </c>
-      <c r="H26" s="1">
+      <c r="Q26" s="1">
         <v>20.35</v>
       </c>
-      <c r="I26" s="1">
+      <c r="R26" s="1">
         <v>20.3</v>
       </c>
-      <c r="J26" s="1">
+      <c r="S26" s="1">
         <v>20.42</v>
       </c>
-      <c r="K26" s="1">
+      <c r="T26" s="1">
         <v>20.36</v>
       </c>
-      <c r="L26" s="1">
+      <c r="U26" s="1">
         <v>20.43</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:21">
       <c r="A27" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B27" s="1">
+        <v>23.63</v>
+      </c>
+      <c r="C27" s="1">
+        <v>23.93</v>
+      </c>
+      <c r="D27" s="1">
+        <v>19.26</v>
+      </c>
+      <c r="E27" s="1">
+        <v>19.02</v>
+      </c>
+      <c r="F27" s="1">
+        <v>19.19</v>
+      </c>
+      <c r="G27" s="1">
+        <v>19.96</v>
+      </c>
+      <c r="H27" s="1">
+        <v>19.87</v>
+      </c>
+      <c r="I27" s="1">
+        <v>20.18</v>
+      </c>
+      <c r="J27" s="1">
+        <v>20.84</v>
+      </c>
+      <c r="K27" s="1">
         <v>21.54</v>
       </c>
-      <c r="C27" s="1">
+      <c r="L27" s="1">
         <v>27.15</v>
       </c>
-      <c r="D27" s="1">
+      <c r="M27" s="1">
         <v>27.89</v>
       </c>
-      <c r="E27" s="1">
+      <c r="N27" s="1">
         <v>27.93</v>
       </c>
-      <c r="F27" s="1">
+      <c r="O27" s="1">
         <v>27.74</v>
       </c>
-      <c r="G27" s="1">
+      <c r="P27" s="1">
         <v>27.69</v>
       </c>
-      <c r="H27" s="1">
+      <c r="Q27" s="1">
         <v>27.85</v>
       </c>
-      <c r="I27" s="1">
+      <c r="R27" s="1">
         <v>27.75</v>
       </c>
-      <c r="J27" s="1">
+      <c r="S27" s="1">
         <v>27.88</v>
       </c>
-      <c r="K27" s="1">
+      <c r="T27" s="1">
         <v>27.89</v>
       </c>
-      <c r="L27" s="1">
+      <c r="U27" s="1">
         <v>27.99</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:21">
       <c r="A29" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B29" s="1">
+        <v>-0.42</v>
+      </c>
+      <c r="C29" s="1">
+        <v>-0.37</v>
+      </c>
+      <c r="D29" s="1">
+        <v>7.56</v>
+      </c>
+      <c r="E29" s="1">
+        <v>6.79</v>
+      </c>
+      <c r="F29" s="1">
+        <v>6.99</v>
+      </c>
+      <c r="G29" s="1">
+        <v>8.42</v>
+      </c>
+      <c r="H29" s="1">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="I29" s="1">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="J29" s="1">
+        <v>8.51</v>
+      </c>
+      <c r="K29" s="1">
         <v>8.15</v>
       </c>
-      <c r="C29" s="1">
+      <c r="L29" s="1">
         <v>1.04</v>
       </c>
-      <c r="D29" s="1">
+      <c r="M29" s="1">
         <v>0.72</v>
       </c>
-      <c r="E29" s="1">
+      <c r="N29" s="1">
         <v>0.64</v>
       </c>
-      <c r="F29" s="1">
+      <c r="O29" s="1">
         <v>0.43</v>
       </c>
-      <c r="G29" s="1">
+      <c r="P29" s="1">
         <v>0.43</v>
       </c>
-      <c r="H29" s="1">
+      <c r="Q29" s="1">
         <v>0.48</v>
       </c>
-      <c r="I29" s="1">
+      <c r="R29" s="1">
         <v>0.27</v>
       </c>
-      <c r="J29" s="1">
+      <c r="S29" s="1">
         <v>0.36</v>
       </c>
-      <c r="K29" s="1">
+      <c r="T29" s="1">
         <v>0.16</v>
       </c>
-      <c r="L29" s="1">
+      <c r="U29" s="1">
         <v>0.16</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:21">
       <c r="A30" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:21">
       <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="1">
+        <v>-2.35</v>
+      </c>
+      <c r="C31" s="1">
+        <v>-2.39</v>
+      </c>
+      <c r="D31" s="1">
+        <v>-0.22</v>
+      </c>
+      <c r="E31" s="1">
+        <v>-0.23</v>
+      </c>
+      <c r="F31" s="1">
+        <v>-0.21</v>
+      </c>
+      <c r="G31" s="1">
+        <v>-0.19</v>
+      </c>
+      <c r="H31" s="1">
         <v>-0.17</v>
       </c>
-      <c r="C31" s="1">
+      <c r="I31" s="1">
+        <v>-0.15</v>
+      </c>
+      <c r="J31" s="1">
+        <v>-0.15</v>
+      </c>
+      <c r="K31" s="1">
+        <v>-0.17</v>
+      </c>
+      <c r="L31" s="1">
         <v>-2.34</v>
       </c>
-      <c r="D31" s="1">
+      <c r="M31" s="1">
         <v>-2.38</v>
       </c>
-      <c r="E31" s="1">
+      <c r="N31" s="1">
         <v>-2.38</v>
       </c>
-      <c r="F31" s="1">
+      <c r="O31" s="1">
         <v>-2.38</v>
       </c>
-      <c r="G31" s="1">
+      <c r="P31" s="1">
         <v>-2.38</v>
       </c>
-      <c r="H31" s="1">
+      <c r="Q31" s="1">
         <v>-2.39</v>
       </c>
-      <c r="I31" s="1">
+      <c r="R31" s="1">
         <v>-2.39</v>
       </c>
-      <c r="J31" s="1">
+      <c r="S31" s="1">
         <v>-2.4</v>
       </c>
-      <c r="K31" s="1">
+      <c r="T31" s="1">
         <v>-2.4</v>
       </c>
-      <c r="L31" s="1">
+      <c r="U31" s="1">
         <v>-2.41</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:21">
       <c r="A32" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B32" s="1">
+        <v>5.07</v>
+      </c>
+      <c r="C32" s="1">
+        <v>5.43</v>
+      </c>
+      <c r="D32" s="1">
+        <v>25.51</v>
+      </c>
+      <c r="E32" s="1">
+        <v>23.26</v>
+      </c>
+      <c r="F32" s="1">
+        <v>23.58</v>
+      </c>
+      <c r="G32" s="1">
+        <v>27.91</v>
+      </c>
+      <c r="H32" s="1">
+        <v>27.77</v>
+      </c>
+      <c r="I32" s="1">
+        <v>28.02</v>
+      </c>
+      <c r="J32" s="1">
+        <v>28.19</v>
+      </c>
+      <c r="K32" s="1">
         <v>27.43</v>
       </c>
-      <c r="C32" s="1">
+      <c r="L32" s="1">
         <v>10.74</v>
       </c>
-      <c r="D32" s="1">
+      <c r="M32" s="1">
         <v>9.710000000000001</v>
       </c>
-      <c r="E32" s="1">
+      <c r="N32" s="1">
         <v>9.4</v>
       </c>
-      <c r="F32" s="1">
+      <c r="O32" s="1">
         <v>8.609999999999999</v>
       </c>
-      <c r="G32" s="1">
+      <c r="P32" s="1">
         <v>8.66</v>
       </c>
-      <c r="H32" s="1">
+      <c r="Q32" s="1">
         <v>8.85</v>
       </c>
-      <c r="I32" s="1">
+      <c r="R32" s="1">
         <v>8.09</v>
       </c>
-      <c r="J32" s="1">
+      <c r="S32" s="1">
         <v>8.44</v>
       </c>
-      <c r="K32" s="1">
+      <c r="T32" s="1">
         <v>7.71</v>
       </c>
-      <c r="L32" s="1">
+      <c r="U32" s="1">
         <v>7.73</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:21">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:21">
       <c r="A35" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B35" s="1">
+        <v>14.34</v>
+      </c>
+      <c r="C35" s="1">
+        <v>14.53</v>
+      </c>
+      <c r="D35" s="1">
+        <v>13.52</v>
+      </c>
+      <c r="E35" s="1">
+        <v>13.03</v>
+      </c>
+      <c r="F35" s="1">
+        <v>13.21</v>
+      </c>
+      <c r="G35" s="1">
+        <v>14.34</v>
+      </c>
+      <c r="H35" s="1">
+        <v>14.3</v>
+      </c>
+      <c r="I35" s="1">
+        <v>14.25</v>
+      </c>
+      <c r="J35" s="1">
+        <v>14.75</v>
+      </c>
+      <c r="K35" s="1">
         <v>15.01</v>
       </c>
-      <c r="C35" s="1">
+      <c r="L35" s="1">
         <v>14.18</v>
       </c>
-      <c r="D35" s="1">
+      <c r="M35" s="1">
         <v>14.58</v>
       </c>
-      <c r="E35" s="1">
+      <c r="N35" s="1">
         <v>14.59</v>
       </c>
-      <c r="F35" s="1">
+      <c r="O35" s="1">
         <v>14.5</v>
       </c>
-      <c r="G35" s="1">
+      <c r="P35" s="1">
         <v>14.59</v>
       </c>
-      <c r="H35" s="1">
+      <c r="Q35" s="1">
         <v>14.71</v>
       </c>
-      <c r="I35" s="1">
+      <c r="R35" s="1">
         <v>14.59</v>
       </c>
-      <c r="J35" s="1">
+      <c r="S35" s="1">
         <v>14.7</v>
       </c>
-      <c r="K35" s="1">
+      <c r="T35" s="1">
         <v>14.61</v>
       </c>
-      <c r="L35" s="1">
+      <c r="U35" s="1">
         <v>14.66</v>
       </c>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:21">
       <c r="A36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="1">
+        <v>24.42</v>
+      </c>
+      <c r="C36" s="1">
+        <v>24.67</v>
+      </c>
+      <c r="D36" s="1">
+        <v>18.28</v>
+      </c>
+      <c r="E36" s="1">
+        <v>18.02</v>
+      </c>
+      <c r="F36" s="1">
+        <v>18.18</v>
+      </c>
+      <c r="G36" s="1">
+        <v>19.08</v>
+      </c>
+      <c r="H36" s="1">
+        <v>19.03</v>
+      </c>
+      <c r="I36" s="1">
+        <v>18.88</v>
+      </c>
+      <c r="J36" s="1">
+        <v>19.7</v>
+      </c>
+      <c r="K36" s="1">
         <v>20.38</v>
       </c>
-      <c r="C36" s="1">
+      <c r="L36" s="1">
         <v>23.34</v>
       </c>
-      <c r="D36" s="1">
+      <c r="M36" s="1">
         <v>24.12</v>
       </c>
-      <c r="E36" s="1">
+      <c r="N36" s="1">
         <v>24.18</v>
       </c>
-      <c r="F36" s="1">
+      <c r="O36" s="1">
         <v>24.16</v>
       </c>
-      <c r="G36" s="1">
+      <c r="P36" s="1">
         <v>24.3</v>
       </c>
-      <c r="H36" s="1">
+      <c r="Q36" s="1">
         <v>24.44</v>
       </c>
-      <c r="I36" s="1">
+      <c r="R36" s="1">
         <v>24.37</v>
       </c>
-      <c r="J36" s="1">
+      <c r="S36" s="1">
         <v>24.49</v>
       </c>
-      <c r="K36" s="1">
+      <c r="T36" s="1">
         <v>24.46</v>
       </c>
-      <c r="L36" s="1">
+      <c r="U36" s="1">
         <v>24.55</v>
       </c>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:21">
       <c r="A37" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B37" s="1">
+        <v>31.59</v>
+      </c>
+      <c r="C37" s="1">
+        <v>31.83</v>
+      </c>
+      <c r="D37" s="1">
+        <v>26.08</v>
+      </c>
+      <c r="E37" s="1">
+        <v>25.81</v>
+      </c>
+      <c r="F37" s="1">
+        <v>26.01</v>
+      </c>
+      <c r="G37" s="1">
+        <v>26.83</v>
+      </c>
+      <c r="H37" s="1">
+        <v>26.52</v>
+      </c>
+      <c r="I37" s="1">
+        <v>26.36</v>
+      </c>
+      <c r="J37" s="1">
+        <v>26.57</v>
+      </c>
+      <c r="K37" s="1">
         <v>26.73</v>
       </c>
-      <c r="C37" s="1">
+      <c r="L37" s="1">
         <v>30.21</v>
       </c>
-      <c r="D37" s="1">
+      <c r="M37" s="1">
         <v>30.29</v>
       </c>
-      <c r="E37" s="1">
+      <c r="N37" s="1">
         <v>30.33</v>
       </c>
-      <c r="F37" s="1">
+      <c r="O37" s="1">
         <v>30.18</v>
       </c>
-      <c r="G37" s="1">
+      <c r="P37" s="1">
         <v>30.16</v>
       </c>
-      <c r="H37" s="1">
+      <c r="Q37" s="1">
         <v>30.31</v>
       </c>
-      <c r="I37" s="1">
+      <c r="R37" s="1">
         <v>30.24</v>
       </c>
-      <c r="J37" s="1">
+      <c r="S37" s="1">
         <v>30.36</v>
       </c>
-      <c r="K37" s="1">
+      <c r="T37" s="1">
         <v>30.35</v>
       </c>
-      <c r="L37" s="1">
+      <c r="U37" s="1">
         <v>30.44</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:21">
       <c r="A38" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B38" s="1">
+        <v>-0.42</v>
+      </c>
+      <c r="C38" s="1">
+        <v>-0.37</v>
+      </c>
+      <c r="D38" s="1">
+        <v>7.56</v>
+      </c>
+      <c r="E38" s="1">
+        <v>6.79</v>
+      </c>
+      <c r="F38" s="1">
+        <v>6.99</v>
+      </c>
+      <c r="G38" s="1">
+        <v>8.42</v>
+      </c>
+      <c r="H38" s="1">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="I38" s="1">
+        <v>8.460000000000001</v>
+      </c>
+      <c r="J38" s="1">
+        <v>8.51</v>
+      </c>
+      <c r="K38" s="1">
         <v>8.15</v>
       </c>
-      <c r="C38" s="1">
+      <c r="L38" s="1">
         <v>1.04</v>
       </c>
-      <c r="D38" s="1">
+      <c r="M38" s="1">
         <v>0.72</v>
       </c>
-      <c r="E38" s="1">
+      <c r="N38" s="1">
         <v>0.64</v>
       </c>
-      <c r="F38" s="1">
+      <c r="O38" s="1">
         <v>0.43</v>
       </c>
-      <c r="G38" s="1">
+      <c r="P38" s="1">
         <v>0.43</v>
       </c>
-      <c r="H38" s="1">
+      <c r="Q38" s="1">
         <v>0.48</v>
       </c>
-      <c r="I38" s="1">
+      <c r="R38" s="1">
         <v>0.27</v>
       </c>
-      <c r="J38" s="1">
+      <c r="S38" s="1">
         <v>0.36</v>
       </c>
-      <c r="K38" s="1">
+      <c r="T38" s="1">
         <v>0.16</v>
       </c>
-      <c r="L38" s="1">
+      <c r="U38" s="1">
         <v>0.16</v>
       </c>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:21">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -1319,13 +1877,22 @@
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
-    </row>
-    <row r="41" spans="1:12">
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
+      <c r="Q40" s="4"/>
+      <c r="R40" s="4"/>
+      <c r="S40" s="4"/>
+      <c r="T40" s="4"/>
+      <c r="U40" s="4"/>
+    </row>
+    <row r="41" spans="1:21">
       <c r="A41" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:21">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -1338,6 +1905,15 @@
       <c r="J45" s="4"/>
       <c r="K45" s="4"/>
       <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4"/>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4"/>
+      <c r="T45" s="4"/>
+      <c r="U45" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update data and code for February 2026 baseline
</commit_message>
<xml_diff>
--- a/captax/data/outputs/Current-Law/comprehensive/supplemental_table_EMTRs_Current-Law_comprehensive.xlsx
+++ b/captax/data/outputs/Current-Law/comprehensive/supplemental_table_EMTRs_Current-Law_comprehensive.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{147AB8DA-EC42-4E18-9913-D34168BF23F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="29880" yWindow="1080" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EMTR on Capital Income" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>Effective Marginal Tax Rates on Capital Income, by Tax Year</t>
   </si>
@@ -89,17 +90,20 @@
   </si>
   <si>
     <t>Data source: Congressional Budget Office.</t>
+  </si>
+  <si>
+    <t>** = between -0.05 percentage points and zero.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0_)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,15 +188,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="166" formatCode="&quot;**&quot;;&quot;**&quot;"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -230,7 +246,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -264,6 +280,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -298,9 +315,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -473,25 +491,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A5:M45"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="65.7109375" customWidth="1"/>
     <col min="2" max="13" width="9.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -505,42 +523,42 @@
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C9" s="5">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D9" s="5">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="E9" s="5">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="F9" s="5">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="G9" s="5">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="H9" s="5">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="I9" s="5">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="J9" s="5">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="K9" s="5">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="L9" s="5">
-        <v>2035</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <v>2036</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -554,759 +572,759 @@
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="1">
-        <v>14.74</v>
+        <v>11.7</v>
       </c>
       <c r="C12" s="1">
-        <v>14.43</v>
+        <v>12.07</v>
       </c>
       <c r="D12" s="1">
-        <v>15.06</v>
+        <v>11.98</v>
       </c>
       <c r="E12" s="1">
-        <v>15.09</v>
+        <v>13.04</v>
       </c>
       <c r="F12" s="1">
-        <v>15.04</v>
+        <v>13.86</v>
       </c>
       <c r="G12" s="1">
-        <v>15.18</v>
+        <v>13.81</v>
       </c>
       <c r="H12" s="1">
-        <v>15.3</v>
+        <v>13.74</v>
       </c>
       <c r="I12" s="1">
-        <v>15.19</v>
+        <v>13.77</v>
       </c>
       <c r="J12" s="1">
-        <v>15.31</v>
+        <v>13.75</v>
       </c>
       <c r="K12" s="1">
-        <v>15.22</v>
+        <v>13.73</v>
       </c>
       <c r="L12" s="1">
-        <v>15.28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <v>13.85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="1">
-        <v>18.5</v>
+        <v>14.38</v>
       </c>
       <c r="C14" s="1">
-        <v>21.28</v>
+        <v>15.1</v>
       </c>
       <c r="D14" s="1">
-        <v>22.28</v>
+        <v>15.15</v>
       </c>
       <c r="E14" s="1">
-        <v>22.36</v>
+        <v>16.96</v>
       </c>
       <c r="F14" s="1">
-        <v>22.38</v>
+        <v>17.16</v>
       </c>
       <c r="G14" s="1">
-        <v>22.57</v>
+        <v>17.2</v>
       </c>
       <c r="H14" s="1">
-        <v>22.71</v>
+        <v>17.22</v>
       </c>
       <c r="I14" s="1">
-        <v>22.64</v>
+        <v>17.29</v>
       </c>
       <c r="J14" s="1">
-        <v>22.76</v>
+        <v>17.329999999999998</v>
       </c>
       <c r="K14" s="1">
-        <v>22.73</v>
+        <v>17.34</v>
       </c>
       <c r="L14" s="1">
-        <v>22.81</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+        <v>17.489999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B16" s="1">
-        <v>12.12</v>
+        <v>3.91</v>
       </c>
       <c r="C16" s="1">
-        <v>15.49</v>
+        <v>5.54</v>
       </c>
       <c r="D16" s="1">
-        <v>18.65</v>
+        <v>5.68</v>
       </c>
       <c r="E16" s="1">
-        <v>18.8</v>
+        <v>5.83</v>
       </c>
       <c r="F16" s="1">
-        <v>18.97</v>
+        <v>6.11</v>
       </c>
       <c r="G16" s="1">
-        <v>19.32</v>
+        <v>6.18</v>
       </c>
       <c r="H16" s="1">
-        <v>19.47</v>
+        <v>6.2</v>
       </c>
       <c r="I16" s="1">
-        <v>19.44</v>
+        <v>6.28</v>
       </c>
       <c r="J16" s="1">
-        <v>19.54</v>
+        <v>6.29</v>
       </c>
       <c r="K16" s="1">
-        <v>19.51</v>
+        <v>6.3</v>
       </c>
       <c r="L16" s="1">
-        <v>19.58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <v>6.42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="1">
-        <v>20.79</v>
+        <v>16.89</v>
       </c>
       <c r="C17" s="1">
-        <v>23.02</v>
+        <v>17.64</v>
       </c>
       <c r="D17" s="1">
-        <v>23.69</v>
+        <v>17.64</v>
       </c>
       <c r="E17" s="1">
-        <v>23.71</v>
+        <v>21.27</v>
       </c>
       <c r="F17" s="1">
-        <v>23.67</v>
+        <v>21.41</v>
       </c>
       <c r="G17" s="1">
-        <v>23.78</v>
+        <v>21.46</v>
       </c>
       <c r="H17" s="1">
-        <v>23.9</v>
+        <v>21.48</v>
       </c>
       <c r="I17" s="1">
-        <v>23.8</v>
+        <v>21.55</v>
       </c>
       <c r="J17" s="1">
-        <v>23.95</v>
+        <v>21.58</v>
       </c>
       <c r="K17" s="1">
-        <v>23.89</v>
+        <v>21.6</v>
       </c>
       <c r="L17" s="1">
-        <v>23.98</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
+        <v>21.74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B18" s="1">
-        <v>23.47</v>
+        <v>23.42</v>
       </c>
       <c r="C18" s="1">
-        <v>27.26</v>
+        <v>23.57</v>
       </c>
       <c r="D18" s="1">
-        <v>27.38</v>
+        <v>23.56</v>
       </c>
       <c r="E18" s="1">
-        <v>27.43</v>
+        <v>23.77</v>
       </c>
       <c r="F18" s="1">
-        <v>27.26</v>
+        <v>23.91</v>
       </c>
       <c r="G18" s="1">
-        <v>27.23</v>
+        <v>23.92</v>
       </c>
       <c r="H18" s="1">
-        <v>27.38</v>
+        <v>23.91</v>
       </c>
       <c r="I18" s="1">
-        <v>27.29</v>
+        <v>23.98</v>
       </c>
       <c r="J18" s="1">
-        <v>27.42</v>
+        <v>24.02</v>
       </c>
       <c r="K18" s="1">
-        <v>27.41</v>
+        <v>24.05</v>
       </c>
       <c r="L18" s="1">
-        <v>27.5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
+        <v>24.22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="1">
-        <v>-16.89</v>
+        <v>-30.09</v>
       </c>
       <c r="C19" s="1">
-        <v>-15.38</v>
+        <v>-28.43</v>
       </c>
       <c r="D19" s="1">
-        <v>-14.92</v>
+        <v>-27.59</v>
       </c>
       <c r="E19" s="1">
-        <v>-14.29</v>
+        <v>-26.64</v>
       </c>
       <c r="F19" s="1">
-        <v>-12.96</v>
+        <v>-25.52</v>
       </c>
       <c r="G19" s="1">
-        <v>-11.22</v>
+        <v>-25.39</v>
       </c>
       <c r="H19" s="1">
-        <v>-10.93</v>
+        <v>-25.33</v>
       </c>
       <c r="I19" s="1">
-        <v>-10.91</v>
+        <v>-25.25</v>
       </c>
       <c r="J19" s="1">
-        <v>-10.8</v>
+        <v>-25.21</v>
       </c>
       <c r="K19" s="1">
-        <v>-10.83</v>
+        <v>-25.2</v>
       </c>
       <c r="L19" s="1">
-        <v>-10.75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
+        <v>-25.03</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="1">
-        <v>22.46</v>
+        <v>15.45</v>
       </c>
       <c r="C20" s="1">
-        <v>25.33</v>
+        <v>15.69</v>
       </c>
       <c r="D20" s="1">
-        <v>27.35</v>
+        <v>15.71</v>
       </c>
       <c r="E20" s="1">
-        <v>27.44</v>
+        <v>15.8</v>
       </c>
       <c r="F20" s="1">
-        <v>27.5</v>
+        <v>15.96</v>
       </c>
       <c r="G20" s="1">
-        <v>27.7</v>
+        <v>16.02</v>
       </c>
       <c r="H20" s="1">
-        <v>27.83</v>
+        <v>16.05</v>
       </c>
       <c r="I20" s="1">
-        <v>27.81</v>
+        <v>16.11</v>
       </c>
       <c r="J20" s="1">
-        <v>27.9</v>
+        <v>16.14</v>
       </c>
       <c r="K20" s="1">
-        <v>27.87</v>
+        <v>16.149999999999999</v>
       </c>
       <c r="L20" s="1">
-        <v>27.93</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
+        <v>16.27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B21" s="1">
-        <v>29.44</v>
+        <v>29.06</v>
       </c>
       <c r="C21" s="1">
-        <v>32.13</v>
+        <v>29.17</v>
       </c>
       <c r="D21" s="1">
-        <v>32.19</v>
+        <v>29.13</v>
       </c>
       <c r="E21" s="1">
-        <v>32.23</v>
+        <v>29.25</v>
       </c>
       <c r="F21" s="1">
-        <v>32.1</v>
+        <v>29.35</v>
       </c>
       <c r="G21" s="1">
-        <v>32.09</v>
+        <v>29.38</v>
       </c>
       <c r="H21" s="1">
-        <v>32.23</v>
+        <v>29.4</v>
       </c>
       <c r="I21" s="1">
-        <v>32.19</v>
+        <v>29.45</v>
       </c>
       <c r="J21" s="1">
-        <v>32.28</v>
+        <v>29.5</v>
       </c>
       <c r="K21" s="1">
-        <v>32.28</v>
+        <v>29.51</v>
       </c>
       <c r="L21" s="1">
-        <v>32.36</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
+        <v>29.65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="1">
-        <v>21.6</v>
+        <v>17.579999999999998</v>
       </c>
       <c r="C23" s="1">
-        <v>24.64</v>
+        <v>18.149999999999999</v>
       </c>
       <c r="D23" s="1">
-        <v>25.55</v>
+        <v>18.16</v>
       </c>
       <c r="E23" s="1">
-        <v>25.57</v>
+        <v>19.940000000000001</v>
       </c>
       <c r="F23" s="1">
-        <v>25.55</v>
+        <v>20.079999999999998</v>
       </c>
       <c r="G23" s="1">
-        <v>25.66</v>
+        <v>20.12</v>
       </c>
       <c r="H23" s="1">
-        <v>25.78</v>
+        <v>20.16</v>
       </c>
       <c r="I23" s="1">
-        <v>25.75</v>
+        <v>20.18</v>
       </c>
       <c r="J23" s="1">
-        <v>25.84</v>
+        <v>20.25</v>
       </c>
       <c r="K23" s="1">
-        <v>25.86</v>
+        <v>20.239999999999998</v>
       </c>
       <c r="L23" s="1">
-        <v>25.92</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
+        <v>20.37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B24" s="1">
-        <v>3.96</v>
+        <v>-0.03</v>
       </c>
       <c r="C24" s="1">
-        <v>4.68</v>
+        <v>1.41</v>
       </c>
       <c r="D24" s="1">
-        <v>6.24</v>
+        <v>1.69</v>
       </c>
       <c r="E24" s="1">
-        <v>6.62</v>
+        <v>3.57</v>
       </c>
       <c r="F24" s="1">
-        <v>6.94</v>
+        <v>4.01</v>
       </c>
       <c r="G24" s="1">
-        <v>7.55</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="H24" s="1">
-        <v>7.8</v>
+        <v>4.04</v>
       </c>
       <c r="I24" s="1">
-        <v>7.5</v>
+        <v>4.32</v>
       </c>
       <c r="J24" s="1">
-        <v>7.82</v>
+        <v>4.1900000000000004</v>
       </c>
       <c r="K24" s="1">
-        <v>7.48</v>
+        <v>4.3</v>
       </c>
       <c r="L24" s="1">
-        <v>7.63</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B26" s="1">
-        <v>17.17</v>
+        <v>12.3</v>
       </c>
       <c r="C26" s="1">
-        <v>18.55</v>
+        <v>13.25</v>
       </c>
       <c r="D26" s="1">
-        <v>19.69</v>
+        <v>13.31</v>
       </c>
       <c r="E26" s="1">
-        <v>19.79</v>
+        <v>15.27</v>
       </c>
       <c r="F26" s="1">
-        <v>19.92</v>
+        <v>15.48</v>
       </c>
       <c r="G26" s="1">
-        <v>20.22</v>
+        <v>15.55</v>
       </c>
       <c r="H26" s="1">
-        <v>20.35</v>
+        <v>15.58</v>
       </c>
       <c r="I26" s="1">
-        <v>20.3</v>
+        <v>15.65</v>
       </c>
       <c r="J26" s="1">
-        <v>20.42</v>
+        <v>15.68</v>
       </c>
       <c r="K26" s="1">
-        <v>20.36</v>
+        <v>15.69</v>
       </c>
       <c r="L26" s="1">
-        <v>20.43</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
+        <v>15.82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B27" s="1">
-        <v>21.54</v>
+        <v>18.96</v>
       </c>
       <c r="C27" s="1">
-        <v>27.15</v>
+        <v>19.22</v>
       </c>
       <c r="D27" s="1">
-        <v>27.89</v>
+        <v>19.25</v>
       </c>
       <c r="E27" s="1">
-        <v>27.93</v>
+        <v>20.74</v>
       </c>
       <c r="F27" s="1">
-        <v>27.74</v>
+        <v>20.92</v>
       </c>
       <c r="G27" s="1">
-        <v>27.69</v>
+        <v>20.91</v>
       </c>
       <c r="H27" s="1">
-        <v>27.85</v>
+        <v>20.88</v>
       </c>
       <c r="I27" s="1">
-        <v>27.75</v>
+        <v>20.96</v>
       </c>
       <c r="J27" s="1">
-        <v>27.88</v>
+        <v>21.01</v>
       </c>
       <c r="K27" s="1">
-        <v>27.89</v>
+        <v>21.03</v>
       </c>
       <c r="L27" s="1">
-        <v>27.99</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+        <v>21.21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B29" s="1">
-        <v>8.15</v>
+        <v>7.14</v>
       </c>
       <c r="C29" s="1">
-        <v>1.04</v>
+        <v>6.84</v>
       </c>
       <c r="D29" s="1">
-        <v>0.72</v>
+        <v>6.47</v>
       </c>
       <c r="E29" s="1">
-        <v>0.64</v>
+        <v>6.04</v>
       </c>
       <c r="F29" s="1">
-        <v>0.43</v>
+        <v>8.08</v>
       </c>
       <c r="G29" s="1">
-        <v>0.43</v>
+        <v>7.87</v>
       </c>
       <c r="H29" s="1">
-        <v>0.48</v>
+        <v>7.63</v>
       </c>
       <c r="I29" s="1">
-        <v>0.27</v>
+        <v>7.59</v>
       </c>
       <c r="J29" s="1">
-        <v>0.36</v>
+        <v>7.43</v>
       </c>
       <c r="K29" s="1">
-        <v>0.16</v>
+        <v>7.36</v>
       </c>
       <c r="L29" s="1">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12">
+        <v>7.43</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B31" s="1">
-        <v>-0.17</v>
+        <v>-0.91</v>
       </c>
       <c r="C31" s="1">
-        <v>-2.34</v>
+        <v>-0.94</v>
       </c>
       <c r="D31" s="1">
-        <v>-2.38</v>
+        <v>-0.98</v>
       </c>
       <c r="E31" s="1">
-        <v>-2.38</v>
+        <v>-1.02</v>
       </c>
       <c r="F31" s="1">
-        <v>-2.38</v>
+        <v>-0.12</v>
       </c>
       <c r="G31" s="1">
-        <v>-2.38</v>
+        <v>-0.12</v>
       </c>
       <c r="H31" s="1">
-        <v>-2.39</v>
+        <v>-0.11</v>
       </c>
       <c r="I31" s="1">
-        <v>-2.39</v>
+        <v>-0.11</v>
       </c>
       <c r="J31" s="1">
-        <v>-2.4</v>
+        <v>-0.11</v>
       </c>
       <c r="K31" s="1">
-        <v>-2.4</v>
+        <v>-0.1</v>
       </c>
       <c r="L31" s="1">
-        <v>-2.41</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B32" s="1">
-        <v>27.43</v>
+        <v>25.57</v>
       </c>
       <c r="C32" s="1">
-        <v>10.74</v>
+        <v>24.87</v>
       </c>
       <c r="D32" s="1">
-        <v>9.710000000000001</v>
+        <v>23.94</v>
       </c>
       <c r="E32" s="1">
-        <v>9.4</v>
+        <v>22.85</v>
       </c>
       <c r="F32" s="1">
-        <v>8.609999999999999</v>
+        <v>26.83</v>
       </c>
       <c r="G32" s="1">
-        <v>8.66</v>
+        <v>26.25</v>
       </c>
       <c r="H32" s="1">
-        <v>8.85</v>
+        <v>25.56</v>
       </c>
       <c r="I32" s="1">
-        <v>8.09</v>
+        <v>25.52</v>
       </c>
       <c r="J32" s="1">
-        <v>8.44</v>
+        <v>25.06</v>
       </c>
       <c r="K32" s="1">
-        <v>7.71</v>
+        <v>24.87</v>
       </c>
       <c r="L32" s="1">
-        <v>7.73</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12">
+        <v>25.11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B35" s="1">
-        <v>15.01</v>
+        <v>12.86</v>
       </c>
       <c r="C35" s="1">
-        <v>14.18</v>
+        <v>13.07</v>
       </c>
       <c r="D35" s="1">
-        <v>14.58</v>
+        <v>12.93</v>
       </c>
       <c r="E35" s="1">
-        <v>14.59</v>
+        <v>13.58</v>
       </c>
       <c r="F35" s="1">
-        <v>14.5</v>
+        <v>14.52</v>
       </c>
       <c r="G35" s="1">
-        <v>14.59</v>
+        <v>14.45</v>
       </c>
       <c r="H35" s="1">
-        <v>14.71</v>
+        <v>14.36</v>
       </c>
       <c r="I35" s="1">
-        <v>14.59</v>
+        <v>14.39</v>
       </c>
       <c r="J35" s="1">
-        <v>14.7</v>
+        <v>14.35</v>
       </c>
       <c r="K35" s="1">
-        <v>14.61</v>
+        <v>14.33</v>
       </c>
       <c r="L35" s="1">
-        <v>14.66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
+        <v>14.45</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B36" s="1">
-        <v>20.38</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="C36" s="1">
-        <v>23.34</v>
+        <v>18</v>
       </c>
       <c r="D36" s="1">
-        <v>24.12</v>
+        <v>18.03</v>
       </c>
       <c r="E36" s="1">
-        <v>24.18</v>
+        <v>19.41</v>
       </c>
       <c r="F36" s="1">
-        <v>24.16</v>
+        <v>19.59</v>
       </c>
       <c r="G36" s="1">
-        <v>24.3</v>
+        <v>19.62</v>
       </c>
       <c r="H36" s="1">
-        <v>24.44</v>
+        <v>19.64</v>
       </c>
       <c r="I36" s="1">
-        <v>24.37</v>
+        <v>19.7</v>
       </c>
       <c r="J36" s="1">
-        <v>24.49</v>
+        <v>19.75</v>
       </c>
       <c r="K36" s="1">
-        <v>24.46</v>
+        <v>19.760000000000002</v>
       </c>
       <c r="L36" s="1">
-        <v>24.55</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
+        <v>19.91</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B37" s="1">
-        <v>26.73</v>
+        <v>26.74</v>
       </c>
       <c r="C37" s="1">
-        <v>30.21</v>
+        <v>26.88</v>
       </c>
       <c r="D37" s="1">
-        <v>30.29</v>
+        <v>26.86</v>
       </c>
       <c r="E37" s="1">
-        <v>30.33</v>
+        <v>27.05</v>
       </c>
       <c r="F37" s="1">
-        <v>30.18</v>
+        <v>27.18</v>
       </c>
       <c r="G37" s="1">
-        <v>30.16</v>
+        <v>27.2</v>
       </c>
       <c r="H37" s="1">
-        <v>30.31</v>
+        <v>27.2</v>
       </c>
       <c r="I37" s="1">
-        <v>30.24</v>
+        <v>27.26</v>
       </c>
       <c r="J37" s="1">
-        <v>30.36</v>
+        <v>27.32</v>
       </c>
       <c r="K37" s="1">
-        <v>30.35</v>
+        <v>27.34</v>
       </c>
       <c r="L37" s="1">
-        <v>30.44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B38" s="1">
-        <v>8.15</v>
+        <v>7.14</v>
       </c>
       <c r="C38" s="1">
-        <v>1.04</v>
+        <v>6.84</v>
       </c>
       <c r="D38" s="1">
-        <v>0.72</v>
+        <v>6.47</v>
       </c>
       <c r="E38" s="1">
-        <v>0.64</v>
+        <v>6.04</v>
       </c>
       <c r="F38" s="1">
-        <v>0.43</v>
+        <v>8.08</v>
       </c>
       <c r="G38" s="1">
-        <v>0.43</v>
+        <v>7.87</v>
       </c>
       <c r="H38" s="1">
-        <v>0.48</v>
+        <v>7.63</v>
       </c>
       <c r="I38" s="1">
-        <v>0.27</v>
+        <v>7.59</v>
       </c>
       <c r="J38" s="1">
-        <v>0.36</v>
+        <v>7.43</v>
       </c>
       <c r="K38" s="1">
-        <v>0.16</v>
+        <v>7.36</v>
       </c>
       <c r="L38" s="1">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12">
+        <v>7.43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -1320,12 +1338,17 @@
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:12">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
@@ -1340,6 +1363,13 @@
       <c r="L45" s="4"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B12:L38">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
+      <formula>-0.049</formula>
+      <formula>-0.001</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>